<commit_message>
fix: two-pass BQ metadata strategy - WIN_NBR and L1_Manager now filled from any row per agent
</commit_message>
<xml_diff>
--- a/Sample Roster.xlsx
+++ b/Sample Roster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://teams.wal-mart.com/sites/CareOps_Centralized_Report/Shared Documents/999. GCP/28.Transportation_Roster_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3907E707-DB11-44F9-983D-D3E49D26616C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{3907E707-DB11-44F9-983D-D3E49D26616C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DEFBD5B-945D-42E4-8342-9C12C7040123}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BDC331FA-51D0-4F18-94AD-B2365784597A}"/>
   </bookViews>
@@ -1091,7 +1091,7 @@
   <dimension ref="A1:AK68"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.7109375" style="9" customWidth="1"/>
     <col min="2" max="2" width="8.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="5" bestFit="1" customWidth="1"/>
@@ -8864,7 +8864,7 @@
         <v>12</v>
       </c>
       <c r="F68" s="5" t="str">
-        <f t="shared" ref="F68:F69" si="4">CONCATENATE(D68," ",E68)</f>
+        <f t="shared" ref="F68" si="4">CONCATENATE(D68," ",E68)</f>
         <v>Pradeep Kutty R</v>
       </c>
       <c r="G68" s="5" t="s">
@@ -9202,15 +9202,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="ac82bdb4-25f0-4a0b-bf0e-699210a12122" xsi:nil="true"/>
@@ -9221,14 +9212,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{690C699D-7F7C-4043-8BF7-3AF13DBC1ADD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{690C699D-7F7C-4043-8BF7-3AF13DBC1ADD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d04923ee-6f79-415f-951a-f07ffe69d73d"/>
+    <ds:schemaRef ds:uri="ac82bdb4-25f0-4a0b-bf0e-699210a12122"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{008001D8-38D3-41C9-B16A-71C42463D52A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17006C0-CF1B-4E33-8A3F-66FA83F6D12A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ac82bdb4-25f0-4a0b-bf0e-699210a12122"/>
+    <ds:schemaRef ds:uri="d04923ee-6f79-415f-951a-f07ffe69d73d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17006C0-CF1B-4E33-8A3F-66FA83F6D12A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{008001D8-38D3-41C9-B16A-71C42463D52A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>